<commit_message>
Ran missing ELDON1 birdNET and added dates for ELDON1 data
</commit_message>
<xml_diff>
--- a/Acoustic_Monitoring/Naming_Cheats.xlsx
+++ b/Acoustic_Monitoring/Naming_Cheats.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rwetz\Documents\GitHub\Acoustic_Monitoring\Acoustic_Monitoring\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6BBB250-E52E-47CE-8106-589204193820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCF69C9C-ABB5-4E85-9B00-4DDE372ABF02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30" yWindow="0" windowWidth="17625" windowHeight="15585" xr2:uid="{3D9CAA4B-74F5-4323-ACD4-E4208151BB44}"/>
+    <workbookView xWindow="-28920" yWindow="555" windowWidth="29040" windowHeight="15720" xr2:uid="{3D9CAA4B-74F5-4323-ACD4-E4208151BB44}"/>
   </bookViews>
   <sheets>
     <sheet name="DATES" sheetId="1" r:id="rId1"/>
-    <sheet name="RECORDERS" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -76,16 +75,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -448,101 +441,131 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{380C074E-5FF2-49B5-BE58-F86B2E186F1C}">
-  <dimension ref="A1:A96"/>
+  <dimension ref="A1:B96"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1">
         <v>20250417</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <f>A1+1</f>
         <v>20250418</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <f t="shared" ref="A3:A14" si="0">A2+1</f>
         <v>20250419</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <f t="shared" si="0"/>
         <v>20250420</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <f t="shared" si="0"/>
         <v>20250421</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <f t="shared" si="0"/>
         <v>20250422</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <f t="shared" si="0"/>
         <v>20250423</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <f t="shared" si="0"/>
         <v>20250424</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <f t="shared" si="0"/>
         <v>20250425</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <f t="shared" si="0"/>
         <v>20250426</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <f t="shared" si="0"/>
         <v>20250427</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <f t="shared" si="0"/>
         <v>20250428</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <f t="shared" si="0"/>
         <v>20250429</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <f t="shared" si="0"/>
         <v>20250430</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>20250501</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <f>A15+1</f>
         <v>20250502</v>
@@ -1029,65 +1052,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87729CED-0C19-4A01-A32F-64BB7A960E06}">
-  <dimension ref="A1:A10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Added code, moved files, added dates
</commit_message>
<xml_diff>
--- a/Acoustic_Monitoring/Naming_Cheats.xlsx
+++ b/Acoustic_Monitoring/Naming_Cheats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rwetz\Documents\GitHub\Acoustic_Monitoring\Acoustic_Monitoring\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCF69C9C-ABB5-4E85-9B00-4DDE372ABF02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{391B1273-655A-4B9A-B6D2-31948371350D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="555" windowWidth="29040" windowHeight="15720" xr2:uid="{3D9CAA4B-74F5-4323-ACD4-E4208151BB44}"/>
+    <workbookView xWindow="-10845" yWindow="675" windowWidth="11010" windowHeight="15585" xr2:uid="{3D9CAA4B-74F5-4323-ACD4-E4208151BB44}"/>
   </bookViews>
   <sheets>
     <sheet name="DATES" sheetId="1" r:id="rId1"/>
@@ -441,610 +441,620 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{380C074E-5FF2-49B5-BE58-F86B2E186F1C}">
-  <dimension ref="A1:B96"/>
+  <dimension ref="A1:B98"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1">
-        <v>20250417</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
+      <c r="A1">
+        <v>20250415</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <f>A1+1</f>
-        <v>20250418</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
+      <c r="A2">
+        <v>20250416</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <f t="shared" ref="A3:A14" si="0">A2+1</f>
-        <v>20250419</v>
+        <v>20250417</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <f t="shared" si="0"/>
-        <v>20250420</v>
+        <f>A3+1</f>
+        <v>20250418</v>
       </c>
       <c r="B4" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <f t="shared" si="0"/>
-        <v>20250421</v>
+        <f t="shared" ref="A5:A16" si="0">A4+1</f>
+        <v>20250419</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <f t="shared" si="0"/>
-        <v>20250422</v>
+        <v>20250420</v>
       </c>
       <c r="B6" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <f t="shared" si="0"/>
-        <v>20250423</v>
+        <v>20250421</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <f t="shared" si="0"/>
-        <v>20250424</v>
+        <v>20250422</v>
       </c>
       <c r="B8" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <f t="shared" si="0"/>
-        <v>20250425</v>
+        <v>20250423</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <f t="shared" si="0"/>
-        <v>20250426</v>
+        <v>20250424</v>
       </c>
       <c r="B10" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <f t="shared" si="0"/>
-        <v>20250427</v>
+        <v>20250425</v>
+      </c>
+      <c r="B11" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <f t="shared" si="0"/>
-        <v>20250428</v>
+        <v>20250426</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <f t="shared" si="0"/>
-        <v>20250429</v>
+        <v>20250427</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <f t="shared" si="0"/>
-        <v>20250430</v>
+        <v>20250428</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>20250501</v>
+      <c r="A15" s="1">
+        <f t="shared" si="0"/>
+        <v>20250429</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <f>A15+1</f>
-        <v>20250502</v>
+        <f t="shared" si="0"/>
+        <v>20250430</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
-        <f t="shared" ref="A17:A45" si="1">A16+1</f>
-        <v>20250503</v>
+      <c r="A17">
+        <v>20250501</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <f t="shared" si="1"/>
-        <v>20250504</v>
+        <f>A17+1</f>
+        <v>20250502</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <f t="shared" si="1"/>
-        <v>20250505</v>
+        <f t="shared" ref="A19:A47" si="1">A18+1</f>
+        <v>20250503</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <f t="shared" si="1"/>
-        <v>20250506</v>
+        <v>20250504</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <f t="shared" si="1"/>
-        <v>20250507</v>
+        <v>20250505</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <f t="shared" si="1"/>
-        <v>20250508</v>
+        <v>20250506</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <f t="shared" si="1"/>
-        <v>20250509</v>
+        <v>20250507</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <f t="shared" si="1"/>
-        <v>20250510</v>
+        <v>20250508</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <f t="shared" si="1"/>
-        <v>20250511</v>
+        <v>20250509</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <f t="shared" si="1"/>
-        <v>20250512</v>
+        <v>20250510</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <f t="shared" si="1"/>
-        <v>20250513</v>
+        <v>20250511</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <f t="shared" si="1"/>
-        <v>20250514</v>
+        <v>20250512</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <f t="shared" si="1"/>
-        <v>20250515</v>
+        <v>20250513</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <f t="shared" si="1"/>
-        <v>20250516</v>
+        <v>20250514</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <f t="shared" si="1"/>
-        <v>20250517</v>
+        <v>20250515</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <f>A31+1</f>
-        <v>20250518</v>
+        <f t="shared" si="1"/>
+        <v>20250516</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <f t="shared" si="1"/>
-        <v>20250519</v>
+        <v>20250517</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <f t="shared" si="1"/>
-        <v>20250520</v>
+        <f>A33+1</f>
+        <v>20250518</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <f t="shared" si="1"/>
-        <v>20250521</v>
+        <v>20250519</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <f t="shared" si="1"/>
-        <v>20250522</v>
+        <v>20250520</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <f t="shared" si="1"/>
-        <v>20250523</v>
+        <v>20250521</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <f t="shared" si="1"/>
-        <v>20250524</v>
+        <v>20250522</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <f t="shared" si="1"/>
-        <v>20250525</v>
+        <v>20250523</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <f t="shared" si="1"/>
-        <v>20250526</v>
+        <v>20250524</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <f t="shared" si="1"/>
-        <v>20250527</v>
+        <v>20250525</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <f t="shared" si="1"/>
-        <v>20250528</v>
+        <v>20250526</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <f t="shared" si="1"/>
-        <v>20250529</v>
+        <v>20250527</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <f t="shared" si="1"/>
-        <v>20250530</v>
+        <v>20250528</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <f t="shared" si="1"/>
-        <v>20250531</v>
+        <v>20250529</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46">
-        <v>20250601</v>
+      <c r="A46" s="1">
+        <f t="shared" si="1"/>
+        <v>20250530</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <f>A46+1</f>
-        <v>20250602</v>
+        <f t="shared" si="1"/>
+        <v>20250531</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" s="1">
-        <f t="shared" ref="A48:A74" si="2">A47+1</f>
-        <v>20250603</v>
+      <c r="A48">
+        <v>20250601</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <f t="shared" si="2"/>
-        <v>20250604</v>
+        <f>A48+1</f>
+        <v>20250602</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <f t="shared" si="2"/>
-        <v>20250605</v>
+        <f t="shared" ref="A50:A76" si="2">A49+1</f>
+        <v>20250603</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <f t="shared" si="2"/>
-        <v>20250606</v>
+        <v>20250604</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <f t="shared" si="2"/>
-        <v>20250607</v>
+        <v>20250605</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <f t="shared" si="2"/>
-        <v>20250608</v>
+        <v>20250606</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <f t="shared" si="2"/>
-        <v>20250609</v>
+        <v>20250607</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <f t="shared" si="2"/>
-        <v>20250610</v>
+        <v>20250608</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <f t="shared" si="2"/>
-        <v>20250611</v>
+        <v>20250609</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <f t="shared" si="2"/>
-        <v>20250612</v>
+        <v>20250610</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <f t="shared" si="2"/>
-        <v>20250613</v>
+        <v>20250611</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <f t="shared" si="2"/>
-        <v>20250614</v>
+        <v>20250612</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <f t="shared" si="2"/>
-        <v>20250615</v>
+        <v>20250613</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <f>A60+1</f>
-        <v>20250616</v>
+        <f t="shared" si="2"/>
+        <v>20250614</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <f t="shared" si="2"/>
-        <v>20250617</v>
+        <v>20250615</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
-        <f t="shared" si="2"/>
-        <v>20250618</v>
+        <f>A62+1</f>
+        <v>20250616</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <f t="shared" si="2"/>
-        <v>20250619</v>
+        <v>20250617</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <f t="shared" si="2"/>
-        <v>20250620</v>
+        <v>20250618</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <f t="shared" si="2"/>
-        <v>20250621</v>
+        <v>20250619</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <f t="shared" si="2"/>
-        <v>20250622</v>
+        <v>20250620</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <f t="shared" si="2"/>
-        <v>20250623</v>
+        <v>20250621</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <f t="shared" si="2"/>
-        <v>20250624</v>
+        <v>20250622</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <f t="shared" si="2"/>
-        <v>20250625</v>
+        <v>20250623</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <f t="shared" si="2"/>
-        <v>20250626</v>
+        <v>20250624</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <f t="shared" si="2"/>
-        <v>20250627</v>
+        <v>20250625</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <f t="shared" si="2"/>
-        <v>20250628</v>
+        <v>20250626</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <f t="shared" si="2"/>
-        <v>20250629</v>
+        <v>20250627</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <f>A74+1</f>
-        <v>20250630</v>
+        <f t="shared" si="2"/>
+        <v>20250628</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A76">
-        <v>20250701</v>
+      <c r="A76" s="1">
+        <f t="shared" si="2"/>
+        <v>20250629</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <f>A76+1</f>
-        <v>20250702</v>
+        <v>20250630</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78" s="1">
-        <f t="shared" ref="A78:A96" si="3">A77+1</f>
-        <v>20250703</v>
+      <c r="A78">
+        <v>20250701</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
-        <f t="shared" si="3"/>
-        <v>20250704</v>
+        <f>A78+1</f>
+        <v>20250702</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
-        <f t="shared" si="3"/>
-        <v>20250705</v>
+        <f t="shared" ref="A80:A98" si="3">A79+1</f>
+        <v>20250703</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <f t="shared" si="3"/>
-        <v>20250706</v>
+        <v>20250704</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <f t="shared" si="3"/>
-        <v>20250707</v>
+        <v>20250705</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <f t="shared" si="3"/>
-        <v>20250708</v>
+        <v>20250706</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <f t="shared" si="3"/>
-        <v>20250709</v>
+        <v>20250707</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <f t="shared" si="3"/>
-        <v>20250710</v>
+        <v>20250708</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <f t="shared" si="3"/>
-        <v>20250711</v>
+        <v>20250709</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <f t="shared" si="3"/>
-        <v>20250712</v>
+        <v>20250710</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <f t="shared" si="3"/>
-        <v>20250713</v>
+        <v>20250711</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <f t="shared" si="3"/>
-        <v>20250714</v>
+        <v>20250712</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <f t="shared" si="3"/>
-        <v>20250715</v>
+        <v>20250713</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <f t="shared" si="3"/>
-        <v>20250716</v>
+        <v>20250714</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <f t="shared" si="3"/>
-        <v>20250717</v>
+        <v>20250715</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <f t="shared" si="3"/>
-        <v>20250718</v>
+        <v>20250716</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <f t="shared" si="3"/>
-        <v>20250719</v>
+        <v>20250717</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
-        <f>A94+1</f>
-        <v>20250720</v>
+        <f t="shared" si="3"/>
+        <v>20250718</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
+        <f t="shared" si="3"/>
+        <v>20250719</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" s="1">
+        <f>A96+1</f>
+        <v>20250720</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" s="1">
         <f t="shared" si="3"/>
         <v>20250721</v>
       </c>

</xml_diff>

<commit_message>
ELDON3 coding & started ELDON4 dates
</commit_message>
<xml_diff>
--- a/Acoustic_Monitoring/Naming_Cheats.xlsx
+++ b/Acoustic_Monitoring/Naming_Cheats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rwetz\Documents\GitHub\Acoustic_Monitoring\Acoustic_Monitoring\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17040E31-4E6B-4033-BB5F-53F66B23BE63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7097EF59-CCA8-4748-9DDB-FE58DC87EF62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-11055" yWindow="675" windowWidth="11175" windowHeight="15585" xr2:uid="{3D9CAA4B-74F5-4323-ACD4-E4208151BB44}"/>
+    <workbookView xWindow="-11235" yWindow="675" windowWidth="11175" windowHeight="15585" xr2:uid="{3D9CAA4B-74F5-4323-ACD4-E4208151BB44}"/>
   </bookViews>
   <sheets>
     <sheet name="DATES" sheetId="1" r:id="rId1"/>
@@ -467,7 +467,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <f>A3+1</f>
+        <f t="shared" ref="A4:A16" si="0">A3+1</f>
         <v>20250418</v>
       </c>
       <c r="B4" t="s">
@@ -476,7 +476,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <f t="shared" ref="A5:A16" si="0">A4+1</f>
+        <f t="shared" si="0"/>
         <v>20250419</v>
       </c>
       <c r="B5" t="s">
@@ -577,13 +577,13 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <f>A17+1</f>
+        <f t="shared" ref="A18:A47" si="1">A17+1</f>
         <v>20250502</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <f t="shared" ref="A19:A47" si="1">A18+1</f>
+        <f t="shared" si="1"/>
         <v>20250503</v>
       </c>
     </row>
@@ -673,7 +673,7 @@
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <f>A33+1</f>
+        <f t="shared" si="1"/>
         <v>20250518</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ELDON4 Dates & code, started ELDON5 Dates
</commit_message>
<xml_diff>
--- a/Acoustic_Monitoring/Naming_Cheats.xlsx
+++ b/Acoustic_Monitoring/Naming_Cheats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rwetz\Documents\GitHub\Acoustic_Monitoring\Acoustic_Monitoring\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7097EF59-CCA8-4748-9DDB-FE58DC87EF62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C9EFB15-2BA3-41C0-A448-8077FF69ED21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-11235" yWindow="675" windowWidth="11175" windowHeight="15585" xr2:uid="{3D9CAA4B-74F5-4323-ACD4-E4208151BB44}"/>
+    <workbookView xWindow="-14505" yWindow="675" windowWidth="14610" windowHeight="15585" xr2:uid="{3D9CAA4B-74F5-4323-ACD4-E4208151BB44}"/>
   </bookViews>
   <sheets>
     <sheet name="DATES" sheetId="1" r:id="rId1"/>

</xml_diff>